<commit_message>
feat(bringup): pin rework, TMP75 temperature, triangle DAC, periodic ADC push
- 引脚重构（app.overlay / pin_config.xlsx / communication_protocol.md）：
  PA12 由 DOUT reg2(pg_13v5) 改为数字输入，PC8-10 三色灯移交 bsp_led；
  DOUT 位图保留 reg 2/4/5/6 空洞以维持后续编号不变（上位机索引稳定）。
- 新增 external/tmp75.[ch]：I2C1(SCL PB8/SDA PB9, WP PB7) 0x48 温度读取，
  12-bit 配置；terminal 增加 temp / i2cscan / i2cread 命令。
- bsp_aout：PA5 输出 0~1.5V、0.25Hz 三角波（0→1.5 锯齿上升、1.5→0 下降往复）。
- sensor：5V0/3V3 通道改用分压系数换算（div2MvFromRaw）。
- terminal：每 1s 周期推送全部 15 路 ADC（默认全通道，无需上位机请求）；
  新增 UART 日志静默接口 terminalIsQuiet()，DFU 升级期间停止一切周期性打印，
  避免打印插进升级协议流（状态机日志同样受其保护）。
- bsp_wtdg：内部 WWDG 窗口 100ms → 1000ms（init 阶段的 TMP75 读取会超出原窗口）。
- bsp_dio：DOUT_FORCE_HIGH_MASK 置空，全部输出交给状态机控制。
- 清理 16 个应用头文件里无意义的 extern "C" 样板（工程为纯 C，无 C++ 编译单元）。
</commit_message>
<xml_diff>
--- a/pin_config.xlsx
+++ b/pin_config.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="30240" windowHeight="12800"/>
+    <workbookView windowWidth="30240" windowHeight="12800" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="241">
   <si>
     <t>ph0</t>
   </si>
@@ -705,6 +706,51 @@
   </si>
   <si>
     <t>is_pc_on</t>
+  </si>
+  <si>
+    <t>PAC1</t>
+  </si>
+  <si>
+    <t>K4_drv</t>
+  </si>
+  <si>
+    <t>PAC2</t>
+  </si>
+  <si>
+    <t>K5_drv</t>
+  </si>
+  <si>
+    <t>PAC3</t>
+  </si>
+  <si>
+    <t>K7_drv</t>
+  </si>
+  <si>
+    <t>PAC4</t>
+  </si>
+  <si>
+    <t>PAC6</t>
+  </si>
+  <si>
+    <t>PDC1</t>
+  </si>
+  <si>
+    <t>PDC2</t>
+  </si>
+  <si>
+    <t>PDC3</t>
+  </si>
+  <si>
+    <t>PDC4</t>
+  </si>
+  <si>
+    <t>PDC5</t>
+  </si>
+  <si>
+    <t>PDC6</t>
+  </si>
+  <si>
+    <t>PDC7</t>
   </si>
 </sst>
 </file>
@@ -1850,7 +1896,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D110"/>
+  <dimension ref="A1:D112"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="3"/>
   <cols>
     <col min="2" max="2" width="23.9230769230769" style="1" customWidth="1"/>
@@ -2859,34 +2905,29 @@
         <v>4</v>
       </c>
     </row>
-    <row r="95" spans="1:3">
-      <c r="A95" t="s">
-        <v>193</v>
-      </c>
-      <c r="B95" t="s">
-        <v>194</v>
-      </c>
-      <c r="C95" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3">
-      <c r="A96" t="s">
-        <v>195</v>
-      </c>
-      <c r="B96" t="s">
-        <v>196</v>
-      </c>
-      <c r="C96" t="s">
-        <v>11</v>
-      </c>
+    <row r="94" spans="1:3">
+      <c r="A94" t="s">
+        <v>175</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C94" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="95" spans="2:2">
+      <c r="B95"/>
+    </row>
+    <row r="96" spans="2:2">
+      <c r="B96"/>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B97" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="C97" t="s">
         <v>11</v>
@@ -2894,10 +2935,10 @@
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="B98" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C98" t="s">
         <v>11</v>
@@ -2905,10 +2946,10 @@
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="B99" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C99" t="s">
         <v>11</v>
@@ -2916,57 +2957,57 @@
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="B100" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C100" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="101" spans="1:4">
+    <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B101" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C101" t="s">
-        <v>4</v>
-      </c>
-      <c r="D101" t="s">
-        <v>207</v>
+        <v>11</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="B102" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C102" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="103" spans="1:3">
+    <row r="103" spans="1:4">
       <c r="A103" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="B103" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C103" t="s">
-        <v>11</v>
+        <v>4</v>
+      </c>
+      <c r="D103" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B104" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="C104" t="s">
         <v>11</v>
@@ -2974,10 +3015,10 @@
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="B105" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="C105" t="s">
         <v>11</v>
@@ -2985,32 +3026,32 @@
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="B106" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="C106" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="B107" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="C107" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B108" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="C108" t="s">
         <v>4</v>
@@ -3018,10 +3059,10 @@
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="B109" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="C109" t="s">
         <v>4</v>
@@ -3029,13 +3070,143 @@
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
+        <v>220</v>
+      </c>
+      <c r="B110" t="s">
+        <v>221</v>
+      </c>
+      <c r="C110" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3">
+      <c r="A111" t="s">
+        <v>222</v>
+      </c>
+      <c r="B111" t="s">
+        <v>223</v>
+      </c>
+      <c r="C111" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3">
+      <c r="A112" t="s">
         <v>224</v>
       </c>
-      <c r="B110" t="s">
+      <c r="B112" t="s">
         <v>225</v>
       </c>
-      <c r="C110" t="s">
+      <c r="C112" t="s">
         <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="1"/>
+  <cols>
+    <col min="2" max="2" width="10.8461538461538" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>226</v>
+      </c>
+      <c r="B1" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>230</v>
+      </c>
+      <c r="B3" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>232</v>
+      </c>
+      <c r="B4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>234</v>
+      </c>
+      <c r="B6" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>235</v>
+      </c>
+      <c r="B7" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>236</v>
+      </c>
+      <c r="B8" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>237</v>
+      </c>
+      <c r="B9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>238</v>
+      </c>
+      <c r="B10" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>239</v>
+      </c>
+      <c r="B11" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>240</v>
+      </c>
+      <c r="B12" t="s">
+        <v>186</v>
       </c>
     </row>
   </sheetData>

</xml_diff>